<commit_message>
updating pubs and people
</commit_message>
<xml_diff>
--- a/source/pages.xlsx
+++ b/source/pages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10107"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harmsm/work/admin/website/website/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C70476-6FFE-4341-9E7C-705199B7A39A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89097B52-B321-8844-ADBF-A0C84C8D1064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34080" yWindow="2540" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{A8B7147D-77A5-1347-9728-F2522D06E352}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{A8B7147D-77A5-1347-9728-F2522D06E352}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="5" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="418">
   <si>
     <t>Evolution of innate immune proteins</t>
   </si>
@@ -74,9 +74,6 @@
     <t>https://github.com/harmsm</t>
   </si>
   <si>
-    <t>https://twitter.com/evolbiochemist</t>
-  </si>
-  <si>
     <t>harms@uoregon.edu</t>
   </si>
   <si>
@@ -1125,6 +1122,174 @@
   </si>
   <si>
     <t>https://ecoevo.social/@EvolBiochemist</t>
+  </si>
+  <si>
+    <t>Brennan Fitzgerald</t>
+  </si>
+  <si>
+    <t>Natalie Jaeger</t>
+  </si>
+  <si>
+    <t>Amelia Kotamarti</t>
+  </si>
+  <si>
+    <t>Post bacc researcher</t>
+  </si>
+  <si>
+    <t>Orlandi K, Phillips S, Harman JL, Sailer ZR, Harms MJ</t>
+  </si>
+  <si>
+    <t>Topiary: a tool for automated high-quality ancestral reconstruction</t>
+  </si>
+  <si>
+    <t>32(2):e4551</t>
+  </si>
+  <si>
+    <t>Chisholm LO, Orlandi KO, Phillips SR, Shavlik MJ, Harms MJ</t>
+  </si>
+  <si>
+    <t>Ancestral reconstruction and the evolution of protein energy landscapes</t>
+  </si>
+  <si>
+    <t>Annual Reviews in Biophysics</t>
+  </si>
+  <si>
+    <t>53:127-146</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1146/annurev-biophys-030722-125440</t>
+  </si>
+  <si>
+    <t>Nixon C, Lim SA, Sternke M, Barrick D, Harms MJ, Marqusee S</t>
+  </si>
+  <si>
+    <t>The importance of input sequence set to consensus-derived proteins and their relationship to reconstructed ancestral proteins</t>
+  </si>
+  <si>
+    <t>33(6):e5011</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1002/pro.5011</t>
+  </si>
+  <si>
+    <t>Garcia A, Shavlik MJ, Harms MJ, Pluth M</t>
+  </si>
+  <si>
+    <t>Structural Deformations in Cucurbit [n] urils: Analysis, Host-Guest Dependence, and Automated Ellipticity Measurements using ElliptiCB [n]</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1002/chem.202401981</t>
+  </si>
+  <si>
+    <t>Tran TTQ, Narayanan C, Loes AN, Click TH, Pham NTH, Létourneau M, Harms MJ, Calmettes C, Agarwal PK, Doucet N</t>
+  </si>
+  <si>
+    <t>Ancestral sequence reconstruction dissects structural and functional differences among eosinophil ribonucleases</t>
+  </si>
+  <si>
+    <t>Journal of Biological Chemistry</t>
+  </si>
+  <si>
+    <t>300(5):107280</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.jbc.2024.107280</t>
+  </si>
+  <si>
+    <t>Glenn SJ, Gentry-Lear Z, Shavlik M, Harms MJ, Asaki TJ, Baylink A</t>
+  </si>
+  <si>
+    <t>Bacterial vampirism mediated through taxis to serum</t>
+  </si>
+  <si>
+    <t>12:RP93178</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7554/eLife.93178.3</t>
+  </si>
+  <si>
+    <t>Orlandi KN, Harms MJ</t>
+  </si>
+  <si>
+    <t>2024.06.25.600640</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1101/2024.06.25.600640</t>
+  </si>
+  <si>
+    <t>Franco K, Gentry-Lear Z, Shavlik M, Harms MJ, Baylink A</t>
+  </si>
+  <si>
+    <t>Navigating contradictions: Salmonella Typhimurium chemotactic responses to conflicting effector stimuli</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7554/eLife.106261.1</t>
+  </si>
+  <si>
+    <t>Svendsen JE, Ford MR, Asnes CL, Oh SC, Dorogin J, Fear KM, O’Hara-Smith JR, Chisholm LO, Phillips SR, Harms MJ, Hosseinzadeh P, Hettiaratchi MH</t>
+  </si>
+  <si>
+    <t>Applying Computational Protein Design to Engineer Affibodies for Affinity-controlled Delivery of Vascular Endothelial Growth Factor and Platelet-Derived Growth Factor</t>
+  </si>
+  <si>
+    <t>Biomacromolecules</t>
+  </si>
+  <si>
+    <t>26(6)</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1021/acs.biomac.5c00097</t>
+  </si>
+  <si>
+    <t>in revision</t>
+  </si>
+  <si>
+    <t>Jaeger NM, Fitzgerald B, Harms MJ</t>
+  </si>
+  <si>
+    <t>Epistasis: Just Say No!</t>
+  </si>
+  <si>
+    <t>Zebrafish do not have a calprotectin ortholog</t>
+  </si>
+  <si>
+    <t>Chemistry-A European Journal</t>
+  </si>
+  <si>
+    <t>30(57):e202401981</t>
+  </si>
+  <si>
+    <t>fitzgerald_circle_150x150.png</t>
+  </si>
+  <si>
+    <t>jaeger_circle_150x150.png</t>
+  </si>
+  <si>
+    <t>akotama2@uoregon.edu</t>
+  </si>
+  <si>
+    <t>njaeger2@uoregon.edu</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/mike-harms-evolbiochemist/</t>
+  </si>
+  <si>
+    <t>bfitzger@uoregon.edu</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>kotamarti_circle_150x150.png</t>
+  </si>
+  <si>
+    <t>How do molecular ensemble shape evolution?</t>
+  </si>
+  <si>
+    <t>High throughput studies of epistasis in transcription factors</t>
+  </si>
+  <si>
+    <t>What is the role of CD14 in S100A9's activation of TLR4?</t>
   </si>
 </sst>
 </file>
@@ -1176,7 +1341,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1185,6 +1350,8 @@
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1204,9 +1371,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1244,7 +1411,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1350,7 +1517,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1492,7 +1659,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1500,7 +1667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDC076B7-4CEB-C143-9E7B-9F55AFCD75D9}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -1514,970 +1681,1191 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C1" t="s">
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C2" t="s">
         <v>268</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="7">
+        <v>2003</v>
+      </c>
+      <c r="E2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F2" t="s">
         <v>269</v>
       </c>
-      <c r="D2">
-        <v>2003</v>
-      </c>
-      <c r="E2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F2" t="s">
-        <v>270</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C3" t="s">
         <v>265</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" s="7">
+        <v>2005</v>
+      </c>
+      <c r="E3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" t="s">
         <v>266</v>
       </c>
-      <c r="D3">
-        <v>2005</v>
-      </c>
-      <c r="E3" t="s">
-        <v>188</v>
-      </c>
-      <c r="F3" t="s">
-        <v>267</v>
-      </c>
       <c r="G3" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B4" t="s">
+        <v>261</v>
+      </c>
+      <c r="C4" t="s">
         <v>262</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="7">
+        <v>2008</v>
+      </c>
+      <c r="E4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F4" t="s">
         <v>263</v>
       </c>
-      <c r="D4">
-        <v>2008</v>
-      </c>
-      <c r="E4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F4" t="s">
-        <v>264</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C5" t="s">
         <v>259</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="7">
+        <v>2009</v>
+      </c>
+      <c r="E5" t="s">
+        <v>242</v>
+      </c>
+      <c r="F5" t="s">
         <v>260</v>
       </c>
-      <c r="D5">
-        <v>2009</v>
-      </c>
-      <c r="E5" t="s">
-        <v>243</v>
-      </c>
-      <c r="F5" t="s">
-        <v>261</v>
-      </c>
       <c r="G5" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D6" s="7">
+        <v>2010</v>
+      </c>
+      <c r="E6" t="s">
+        <v>214</v>
+      </c>
+      <c r="F6" t="s">
         <v>257</v>
       </c>
-      <c r="D6">
-        <v>2010</v>
-      </c>
-      <c r="E6" t="s">
-        <v>215</v>
-      </c>
-      <c r="F6" t="s">
-        <v>258</v>
-      </c>
       <c r="G6" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B7" t="s">
+        <v>254</v>
+      </c>
+      <c r="C7" t="s">
+        <v>253</v>
+      </c>
+      <c r="D7" s="7">
+        <v>2010</v>
+      </c>
+      <c r="E7" t="s">
+        <v>225</v>
+      </c>
+      <c r="F7" t="s">
         <v>255</v>
       </c>
-      <c r="C7" t="s">
-        <v>254</v>
-      </c>
-      <c r="D7">
-        <v>2010</v>
-      </c>
-      <c r="E7" t="s">
-        <v>226</v>
-      </c>
-      <c r="F7" t="s">
-        <v>256</v>
-      </c>
       <c r="G7" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C8" t="s">
         <v>251</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="7">
+        <v>2011</v>
+      </c>
+      <c r="E8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F8" t="s">
         <v>252</v>
       </c>
-      <c r="D8">
-        <v>2011</v>
-      </c>
-      <c r="E8" t="s">
-        <v>188</v>
-      </c>
-      <c r="F8" t="s">
-        <v>253</v>
-      </c>
       <c r="G8" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B9" t="s">
+        <v>248</v>
+      </c>
+      <c r="C9" t="s">
+        <v>245</v>
+      </c>
+      <c r="D9" s="7">
+        <v>2012</v>
+      </c>
+      <c r="E9" t="s">
+        <v>246</v>
+      </c>
+      <c r="F9" t="s">
+        <v>247</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="C9" t="s">
-        <v>246</v>
-      </c>
-      <c r="D9">
-        <v>2012</v>
-      </c>
-      <c r="E9" t="s">
-        <v>247</v>
-      </c>
-      <c r="F9" t="s">
-        <v>248</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B10" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" t="s">
+        <v>240</v>
+      </c>
+      <c r="D10" s="7">
+        <v>2013</v>
+      </c>
+      <c r="E10" t="s">
         <v>242</v>
       </c>
-      <c r="C10" t="s">
-        <v>241</v>
-      </c>
-      <c r="D10">
-        <v>2013</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>243</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C11" t="s">
+        <v>236</v>
+      </c>
+      <c r="D11" s="7">
+        <v>2013</v>
+      </c>
+      <c r="E11" t="s">
         <v>237</v>
       </c>
-      <c r="D11">
-        <v>2013</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>238</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" s="1" t="s">
         <v>239</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B12" t="s">
+        <v>233</v>
+      </c>
+      <c r="C12" t="s">
         <v>234</v>
       </c>
-      <c r="C12" t="s">
-        <v>235</v>
-      </c>
-      <c r="D12">
+      <c r="D12" s="7">
         <v>2013</v>
       </c>
       <c r="E12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B13" t="s">
+        <v>227</v>
+      </c>
+      <c r="C13" t="s">
+        <v>226</v>
+      </c>
+      <c r="D13" s="7">
+        <v>2014</v>
+      </c>
+      <c r="E13" t="s">
         <v>228</v>
       </c>
-      <c r="C13" t="s">
-        <v>227</v>
-      </c>
-      <c r="D13">
-        <v>2014</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>229</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" s="1" t="s">
         <v>230</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B14" t="s">
+        <v>222</v>
+      </c>
+      <c r="C14" t="s">
         <v>223</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" s="7">
+        <v>2014</v>
+      </c>
+      <c r="E14" t="s">
+        <v>225</v>
+      </c>
+      <c r="F14" t="s">
         <v>224</v>
       </c>
-      <c r="D14">
-        <v>2014</v>
-      </c>
-      <c r="E14" t="s">
-        <v>226</v>
-      </c>
-      <c r="F14" t="s">
-        <v>225</v>
-      </c>
       <c r="G14" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B15" t="s">
+        <v>212</v>
+      </c>
+      <c r="C15" t="s">
         <v>213</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="7">
+        <v>2016</v>
+      </c>
+      <c r="E15" t="s">
         <v>214</v>
       </c>
-      <c r="D15">
-        <v>2016</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>215</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B16" t="s">
+        <v>204</v>
+      </c>
+      <c r="C16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D16" s="7">
+        <v>2016</v>
+      </c>
+      <c r="E16" t="s">
+        <v>187</v>
+      </c>
+      <c r="F16" t="s">
         <v>205</v>
       </c>
-      <c r="C16" t="s">
-        <v>204</v>
-      </c>
-      <c r="D16">
-        <v>2016</v>
-      </c>
-      <c r="E16" t="s">
-        <v>188</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B17" t="s">
+        <v>199</v>
+      </c>
+      <c r="C17" t="s">
+        <v>198</v>
+      </c>
+      <c r="D17" s="7">
+        <v>2016</v>
+      </c>
+      <c r="E17" t="s">
         <v>200</v>
       </c>
-      <c r="C17" t="s">
-        <v>199</v>
-      </c>
-      <c r="D17">
-        <v>2016</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>201</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B18" t="s">
+        <v>217</v>
+      </c>
+      <c r="C18" t="s">
         <v>218</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" s="7">
+        <v>2017</v>
+      </c>
+      <c r="E18" t="s">
         <v>219</v>
       </c>
-      <c r="D18">
-        <v>2017</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>220</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B19" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C19" t="s">
+        <v>194</v>
+      </c>
+      <c r="D19" s="7">
+        <v>2017</v>
+      </c>
+      <c r="E19" t="s">
         <v>195</v>
       </c>
-      <c r="D19">
-        <v>2017</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>196</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C20" t="s">
+        <v>191</v>
+      </c>
+      <c r="D20" s="7">
+        <v>2017</v>
+      </c>
+      <c r="E20" t="s">
         <v>192</v>
       </c>
-      <c r="D20">
-        <v>2017</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="G20" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B21" t="s">
+        <v>186</v>
+      </c>
+      <c r="C21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D21" s="7">
+        <v>2017</v>
+      </c>
+      <c r="E21" t="s">
         <v>187</v>
       </c>
-      <c r="C21" t="s">
-        <v>186</v>
-      </c>
-      <c r="D21">
-        <v>2017</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>188</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B22" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C22" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" s="7">
+        <v>2017</v>
+      </c>
+      <c r="E22" t="s">
         <v>182</v>
       </c>
-      <c r="D22">
-        <v>2017</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="F22" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="G22" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B23" t="s">
+        <v>210</v>
+      </c>
+      <c r="C23" t="s">
+        <v>207</v>
+      </c>
+      <c r="D23" s="7">
+        <v>2018</v>
+      </c>
+      <c r="E23" t="s">
+        <v>208</v>
+      </c>
+      <c r="F23" t="s">
+        <v>209</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="C23" t="s">
-        <v>208</v>
-      </c>
-      <c r="D23">
-        <v>2018</v>
-      </c>
-      <c r="E23" t="s">
-        <v>209</v>
-      </c>
-      <c r="F23" t="s">
-        <v>210</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B24" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C24" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="7">
+        <v>2018</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
         <v>179</v>
       </c>
-      <c r="D24">
-        <v>2018</v>
-      </c>
-      <c r="E24" t="s">
-        <v>34</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B25" t="s">
+        <v>175</v>
+      </c>
+      <c r="C25" t="s">
+        <v>174</v>
+      </c>
+      <c r="D25" s="7">
+        <v>2018</v>
+      </c>
+      <c r="E25" t="s">
         <v>176</v>
       </c>
-      <c r="C25" t="s">
-        <v>175</v>
-      </c>
-      <c r="D25">
-        <v>2018</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="G25" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B26" t="s">
+        <v>171</v>
+      </c>
+      <c r="C26" t="s">
+        <v>170</v>
+      </c>
+      <c r="D26" s="7">
+        <v>2018</v>
+      </c>
+      <c r="E26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" t="s">
         <v>172</v>
       </c>
-      <c r="C26" t="s">
-        <v>171</v>
-      </c>
-      <c r="D26">
-        <v>2018</v>
-      </c>
-      <c r="E26" t="s">
-        <v>34</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B27" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" t="s">
         <v>165</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" s="7">
+        <v>2019</v>
+      </c>
+      <c r="E27" t="s">
         <v>166</v>
       </c>
-      <c r="D27">
-        <v>2019</v>
-      </c>
-      <c r="E27" t="s">
-        <v>167</v>
-      </c>
       <c r="F27" t="s">
+        <v>168</v>
+      </c>
+      <c r="G27" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C28" t="s">
-        <v>151</v>
-      </c>
-      <c r="D28">
+        <v>150</v>
+      </c>
+      <c r="D28" s="7">
         <v>2019</v>
       </c>
       <c r="E28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G28" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>303</v>
+      </c>
+      <c r="B29" t="s">
         <v>304</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>305</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" s="7">
+        <v>2019</v>
+      </c>
+      <c r="E29" t="s">
+        <v>148</v>
+      </c>
+      <c r="G29" t="s">
         <v>306</v>
-      </c>
-      <c r="D29">
-        <v>2019</v>
-      </c>
-      <c r="E29" t="s">
-        <v>149</v>
-      </c>
-      <c r="G29" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>160</v>
+      </c>
+      <c r="B30" t="s">
+        <v>159</v>
+      </c>
+      <c r="C30" t="s">
+        <v>158</v>
+      </c>
+      <c r="D30" s="7">
+        <v>2020</v>
+      </c>
+      <c r="E30" t="s">
         <v>161</v>
       </c>
-      <c r="B30" t="s">
-        <v>160</v>
-      </c>
-      <c r="C30" t="s">
-        <v>159</v>
-      </c>
-      <c r="D30">
-        <v>2020</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>162</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B31" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C31" t="s">
-        <v>157</v>
-      </c>
-      <c r="D31">
+        <v>156</v>
+      </c>
+      <c r="D31" s="7">
         <v>2020</v>
       </c>
       <c r="E31" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F31" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C32" t="s">
-        <v>154</v>
-      </c>
-      <c r="D32">
+        <v>153</v>
+      </c>
+      <c r="D32" s="7">
         <v>2020</v>
       </c>
       <c r="E32" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F32" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C33" t="s">
-        <v>155</v>
-      </c>
-      <c r="D33">
+        <v>154</v>
+      </c>
+      <c r="D33" s="7">
         <v>2021</v>
       </c>
       <c r="E33" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B34" t="s">
+        <v>145</v>
+      </c>
+      <c r="C34" t="s">
         <v>146</v>
       </c>
-      <c r="C34" t="s">
-        <v>147</v>
-      </c>
-      <c r="D34">
+      <c r="D34" s="7">
         <v>2021</v>
       </c>
       <c r="E34" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F34" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B35" t="s">
+        <v>283</v>
+      </c>
+      <c r="C35" t="s">
         <v>284</v>
       </c>
-      <c r="C35" t="s">
-        <v>285</v>
-      </c>
-      <c r="D35">
+      <c r="D35" s="7">
         <v>2021</v>
       </c>
       <c r="E35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F35" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B36" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C36" t="s">
-        <v>303</v>
-      </c>
-      <c r="D36">
+        <v>302</v>
+      </c>
+      <c r="D36" s="7">
         <v>2021</v>
       </c>
       <c r="E36" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B37" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C37" t="s">
+        <v>317</v>
+      </c>
+      <c r="D37" s="7">
+        <v>2021</v>
+      </c>
+      <c r="E37" t="s">
+        <v>187</v>
+      </c>
+      <c r="F37" t="s">
+        <v>320</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="D37">
-        <v>2021</v>
-      </c>
-      <c r="E37" t="s">
-        <v>188</v>
-      </c>
-      <c r="F37" t="s">
-        <v>321</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B38" t="s">
+        <v>291</v>
+      </c>
+      <c r="C38" t="s">
         <v>292</v>
       </c>
-      <c r="C38" t="s">
-        <v>293</v>
-      </c>
-      <c r="D38">
+      <c r="D38" s="7">
         <v>2021</v>
       </c>
       <c r="E38" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F38" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B39" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C39" t="s">
-        <v>348</v>
-      </c>
-      <c r="D39">
+        <v>347</v>
+      </c>
+      <c r="D39" s="7">
         <v>2022</v>
       </c>
       <c r="E39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F39" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B40" t="s">
+        <v>352</v>
+      </c>
+      <c r="C40" t="s">
+        <v>351</v>
+      </c>
+      <c r="D40" s="7">
+        <v>2022</v>
+      </c>
+      <c r="E40" t="s">
+        <v>166</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>353</v>
-      </c>
-      <c r="C40" t="s">
-        <v>352</v>
-      </c>
-      <c r="D40">
-        <v>2022</v>
-      </c>
-      <c r="E40" t="s">
-        <v>167</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B41" t="s">
+        <v>354</v>
+      </c>
+      <c r="C41" t="s">
         <v>355</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" s="7">
+        <v>2022</v>
+      </c>
+      <c r="E41" t="s">
         <v>356</v>
       </c>
-      <c r="D41">
-        <v>2022</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>357</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B42" t="s">
+        <v>338</v>
+      </c>
+      <c r="C42" t="s">
         <v>339</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" s="7">
+        <v>2022</v>
+      </c>
+      <c r="E42" t="s">
+        <v>359</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="D42">
-        <v>2022</v>
-      </c>
-      <c r="E42" t="s">
-        <v>360</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C43" t="s">
-        <v>343</v>
-      </c>
-      <c r="D43">
+        <v>342</v>
+      </c>
+      <c r="D43" s="7">
         <v>2022</v>
       </c>
       <c r="E43" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>160</v>
+      </c>
+      <c r="B44" t="s">
+        <v>366</v>
+      </c>
+      <c r="C44" t="s">
+        <v>367</v>
+      </c>
+      <c r="D44" s="7">
+        <v>2023</v>
+      </c>
+      <c r="E44" t="s">
+        <v>166</v>
+      </c>
+      <c r="F44" t="s">
+        <v>368</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>160</v>
+      </c>
+      <c r="B45" t="s">
+        <v>369</v>
+      </c>
+      <c r="C45" t="s">
+        <v>370</v>
+      </c>
+      <c r="D45" s="7">
+        <v>2024</v>
+      </c>
+      <c r="E45" t="s">
+        <v>371</v>
+      </c>
+      <c r="F45" t="s">
+        <v>372</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>160</v>
+      </c>
+      <c r="B46" t="s">
+        <v>374</v>
+      </c>
+      <c r="C46" t="s">
+        <v>375</v>
+      </c>
+      <c r="D46" s="7">
+        <v>2024</v>
+      </c>
+      <c r="E46" t="s">
+        <v>166</v>
+      </c>
+      <c r="F46" t="s">
+        <v>376</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>160</v>
+      </c>
+      <c r="B47" t="s">
+        <v>378</v>
+      </c>
+      <c r="C47" t="s">
+        <v>379</v>
+      </c>
+      <c r="D47" s="7">
+        <v>2024</v>
+      </c>
+      <c r="E47" t="s">
+        <v>405</v>
+      </c>
+      <c r="F47" t="s">
+        <v>406</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>160</v>
+      </c>
+      <c r="B48" t="s">
+        <v>381</v>
+      </c>
+      <c r="C48" t="s">
+        <v>382</v>
+      </c>
+      <c r="D48" s="7">
+        <v>2024</v>
+      </c>
+      <c r="E48" t="s">
+        <v>383</v>
+      </c>
+      <c r="F48" t="s">
+        <v>384</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>160</v>
+      </c>
+      <c r="B49" t="s">
+        <v>386</v>
+      </c>
+      <c r="C49" t="s">
+        <v>387</v>
+      </c>
+      <c r="D49" s="7">
+        <v>2024</v>
+      </c>
+      <c r="E49" t="s">
+        <v>161</v>
+      </c>
+      <c r="F49" t="s">
+        <v>388</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>160</v>
+      </c>
+      <c r="B50" t="s">
+        <v>390</v>
+      </c>
+      <c r="C50" t="s">
+        <v>404</v>
+      </c>
+      <c r="D50" s="7">
+        <v>2025</v>
+      </c>
+      <c r="E50" t="s">
+        <v>200</v>
+      </c>
+      <c r="F50" t="s">
+        <v>391</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>160</v>
+      </c>
+      <c r="B51" t="s">
+        <v>393</v>
+      </c>
+      <c r="C51" t="s">
+        <v>394</v>
+      </c>
+      <c r="D51" s="7">
+        <v>2025</v>
+      </c>
+      <c r="E51" t="s">
+        <v>161</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>160</v>
+      </c>
+      <c r="B52" t="s">
+        <v>396</v>
+      </c>
+      <c r="C52" t="s">
+        <v>397</v>
+      </c>
+      <c r="D52" s="7">
+        <v>2025</v>
+      </c>
+      <c r="E52" t="s">
+        <v>398</v>
+      </c>
+      <c r="F52" t="s">
+        <v>399</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>401</v>
+      </c>
+      <c r="B53" t="s">
+        <v>402</v>
+      </c>
+      <c r="C53" t="s">
+        <v>403</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="E53" t="s">
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -2522,6 +2910,15 @@
     <hyperlink ref="G40" r:id="rId38" xr:uid="{D121D190-6997-DE49-B711-B0A0F985B6AC}"/>
     <hyperlink ref="G42" r:id="rId39" xr:uid="{79020FD8-1031-EE4E-AD55-E6B083D09D45}"/>
     <hyperlink ref="G43" r:id="rId40" xr:uid="{22036C22-E126-FF4D-B5AB-64C14DF4FB9F}"/>
+    <hyperlink ref="G44" r:id="rId41" xr:uid="{C2C45C7B-B8F3-C94C-A49C-37349257F97D}"/>
+    <hyperlink ref="G45" r:id="rId42" xr:uid="{14E0775A-2ADB-C54D-9630-4321E413B703}"/>
+    <hyperlink ref="G46" r:id="rId43" xr:uid="{090EA4C1-31ED-C649-B44E-0FFE29035C52}"/>
+    <hyperlink ref="G47" r:id="rId44" xr:uid="{714605BE-9BAA-AC49-8368-19DCDD41CAD8}"/>
+    <hyperlink ref="G48" r:id="rId45" xr:uid="{D55FF453-A6DC-8B40-B3D0-2C1CD20618A1}"/>
+    <hyperlink ref="G49" r:id="rId46" xr:uid="{2BED8AB7-E75A-D244-9BFE-BC5BDBCBCCA7}"/>
+    <hyperlink ref="G50" r:id="rId47" xr:uid="{E586EEAB-2182-A14F-BF62-4562E07951D6}"/>
+    <hyperlink ref="G51" r:id="rId48" xr:uid="{12648E16-FA8D-EB45-9098-E315041E8C33}"/>
+    <hyperlink ref="G52" r:id="rId49" xr:uid="{E09BF139-DB12-0649-8ED0-408B80AB8425}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2529,7 +2926,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A604AB1-DDFC-4B40-85A4-D0BC5335EE4C}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -2546,7 +2943,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2564,7 +2961,7 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -2573,15 +2970,15 @@
         <v>7</v>
       </c>
       <c r="J1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2593,156 +2990,156 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="H2" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" t="s">
-        <v>13</v>
+      <c r="K2" s="1" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>336</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>110</v>
+        <v>349</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+        <v>343</v>
+      </c>
       <c r="I3" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="J3" s="1"/>
+        <v>344</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>362</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>415</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
-      </c>
+        <v>407</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
       <c r="I4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>298</v>
+        <v>363</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>299</v>
+        <v>416</v>
       </c>
       <c r="E5" t="s">
-        <v>300</v>
-      </c>
+        <v>408</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
       <c r="I5" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>302</v>
+        <v>410</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>364</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>365</v>
       </c>
       <c r="D6" t="s">
-        <v>106</v>
+        <v>417</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
-      </c>
+        <v>414</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
       <c r="I6" s="1" t="s">
-        <v>99</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>101</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="F7" s="1"/>
       <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
       <c r="I7" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>109</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>295</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>102</v>
+        <v>20</v>
+      </c>
+      <c r="J8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -2750,434 +3147,507 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>337</v>
+        <v>297</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>350</v>
+        <v>298</v>
       </c>
       <c r="E9" t="s">
-        <v>344</v>
+        <v>299</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>345</v>
+        <v>300</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>294</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>295</v>
+        <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>296</v>
+        <v>76</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>297</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" t="s">
         <v>14</v>
       </c>
-      <c r="C11" t="s">
-        <v>331</v>
-      </c>
       <c r="D11" t="s">
-        <v>332</v>
+        <v>106</v>
       </c>
       <c r="E11" t="s">
-        <v>74</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>16</v>
+        <v>78</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G11" s="1"/>
+      <c r="I11" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>329</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>330</v>
+        <v>294</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>79</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>293</v>
       </c>
       <c r="C13" t="s">
-        <v>329</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>323</v>
+        <v>294</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>295</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>330</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>331</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G14" s="1"/>
+        <v>73</v>
+      </c>
       <c r="H14" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>105</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>328</v>
       </c>
       <c r="D15" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E15" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
-        <v>33</v>
+        <v>328</v>
       </c>
       <c r="D16" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="s">
         <v>29</v>
       </c>
-      <c r="B17" t="s">
-        <v>37</v>
-      </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
-      </c>
-      <c r="I17" t="s">
-        <v>71</v>
+        <v>82</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
-        <v>279</v>
+        <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>287</v>
+        <v>323</v>
       </c>
       <c r="E18" t="s">
-        <v>72</v>
-      </c>
-      <c r="F18" t="s">
-        <v>60</v>
-      </c>
-      <c r="H18" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" t="s">
-        <v>40</v>
+        <v>324</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>83</v>
+      </c>
+      <c r="I20" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>278</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>286</v>
       </c>
       <c r="E21" t="s">
-        <v>89</v>
+        <v>71</v>
+      </c>
+      <c r="F21" t="s">
+        <v>59</v>
+      </c>
+      <c r="H21" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D22" t="s">
-        <v>286</v>
+        <v>39</v>
       </c>
       <c r="E22" t="s">
-        <v>90</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G22" s="2"/>
-      <c r="H22" t="s">
-        <v>63</v>
-      </c>
-      <c r="I22" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" t="s">
-        <v>326</v>
+        <v>56</v>
       </c>
       <c r="E23" t="s">
-        <v>91</v>
-      </c>
-      <c r="H23" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E24" t="s">
-        <v>92</v>
-      </c>
-      <c r="F24" t="s">
-        <v>66</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>327</v>
+        <v>285</v>
       </c>
       <c r="E25" t="s">
-        <v>93</v>
+        <v>89</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" t="s">
+        <v>62</v>
+      </c>
+      <c r="I25" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D26" t="s">
-        <v>52</v>
+        <v>325</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>90</v>
+      </c>
+      <c r="H26" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C27" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="E27" t="s">
-        <v>95</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G27" s="1"/>
-      <c r="H27" t="s">
-        <v>69</v>
+        <v>91</v>
+      </c>
+      <c r="F27" t="s">
+        <v>65</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D28" t="s">
-        <v>40</v>
+        <v>326</v>
       </c>
       <c r="E28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" t="s">
+        <v>51</v>
+      </c>
+      <c r="E29" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" t="s">
+        <v>32</v>
+      </c>
+      <c r="D30" t="s">
         <v>33</v>
       </c>
-      <c r="D29" t="s">
-        <v>328</v>
-      </c>
-      <c r="E29" t="s">
-        <v>97</v>
-      </c>
-      <c r="F29" t="s">
-        <v>70</v>
+      <c r="E30" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G30" s="1"/>
+      <c r="H30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" t="s">
+        <v>32</v>
+      </c>
+      <c r="D31" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" t="s">
+        <v>32</v>
+      </c>
+      <c r="D32" t="s">
+        <v>327</v>
+      </c>
+      <c r="E32" t="s">
+        <v>96</v>
+      </c>
+      <c r="F32" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{1DE0CD26-AAF6-C14D-AC57-1E20477BBEF9}"/>
-    <hyperlink ref="H2" r:id="rId2" xr:uid="{4B69F9D1-9BDC-3B49-95D5-B892E0F38E93}"/>
-    <hyperlink ref="H11" r:id="rId3" xr:uid="{F297B546-961A-904C-8B57-270571840D4C}"/>
-    <hyperlink ref="I4" r:id="rId4" xr:uid="{82F2EFE6-4E28-F34E-B218-DAA2AC17ECFE}"/>
-    <hyperlink ref="H24" r:id="rId5" xr:uid="{B5F9801A-D1FF-F945-B5EA-A95297A9AC9E}"/>
-    <hyperlink ref="F27" r:id="rId6" xr:uid="{7C843EC2-4C8D-4641-BB36-2B0270ADEE55}"/>
-    <hyperlink ref="I3" r:id="rId7" xr:uid="{B1C6FFD0-CEC7-F545-85D8-C469FD54EC40}"/>
-    <hyperlink ref="I6" r:id="rId8" xr:uid="{0B982E49-986A-0941-8C32-ADEAA21D9033}"/>
-    <hyperlink ref="I7" r:id="rId9" xr:uid="{82A7CA40-D4B3-CD48-B0DD-40DB2C17FB15}"/>
-    <hyperlink ref="F7" r:id="rId10" xr:uid="{DBABC5AF-727A-5F45-976D-9D37304F647C}"/>
-    <hyperlink ref="I8" r:id="rId11" xr:uid="{D81BC1A6-DB5E-2442-8092-0DCC05080E7B}"/>
-    <hyperlink ref="F14" r:id="rId12" xr:uid="{671646BC-4048-784B-A41A-EE3B6A5872DF}"/>
-    <hyperlink ref="H14" r:id="rId13" xr:uid="{520C3AB8-D98F-5A41-A791-18E65C05A26D}"/>
-    <hyperlink ref="I14" r:id="rId14" xr:uid="{AC194642-8CCA-D045-8B43-2E593C852C84}"/>
-    <hyperlink ref="K7" r:id="rId15" xr:uid="{7AD87150-852A-EC48-8A33-35899592670A}"/>
-    <hyperlink ref="I10" r:id="rId16" display="mailto:Jyin5@uoregon.edu" xr:uid="{BD89C2C8-01DA-0945-8C45-44FC2597E1A0}"/>
-    <hyperlink ref="I5" r:id="rId17" display="mailto:konao@uoregon.edu" xr:uid="{99A77FB4-F7EA-7A4E-A1D6-82B0846E355F}"/>
-    <hyperlink ref="K5" r:id="rId18" xr:uid="{72314501-811D-D043-997F-E392845F576D}"/>
-    <hyperlink ref="I9" r:id="rId19" xr:uid="{3B7DC98F-564E-8040-ABB3-24351F91CBD2}"/>
-    <hyperlink ref="G2" r:id="rId20" xr:uid="{944B277E-1502-DF4C-99EE-2856B2C13CD9}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{F297B546-961A-904C-8B57-270571840D4C}"/>
+    <hyperlink ref="I8" r:id="rId3" xr:uid="{82F2EFE6-4E28-F34E-B218-DAA2AC17ECFE}"/>
+    <hyperlink ref="H27" r:id="rId4" xr:uid="{B5F9801A-D1FF-F945-B5EA-A95297A9AC9E}"/>
+    <hyperlink ref="F30" r:id="rId5" xr:uid="{7C843EC2-4C8D-4641-BB36-2B0270ADEE55}"/>
+    <hyperlink ref="I7" r:id="rId6" xr:uid="{B1C6FFD0-CEC7-F545-85D8-C469FD54EC40}"/>
+    <hyperlink ref="I10" r:id="rId7" xr:uid="{0B982E49-986A-0941-8C32-ADEAA21D9033}"/>
+    <hyperlink ref="I11" r:id="rId8" xr:uid="{82A7CA40-D4B3-CD48-B0DD-40DB2C17FB15}"/>
+    <hyperlink ref="F11" r:id="rId9" xr:uid="{DBABC5AF-727A-5F45-976D-9D37304F647C}"/>
+    <hyperlink ref="I12" r:id="rId10" xr:uid="{D81BC1A6-DB5E-2442-8092-0DCC05080E7B}"/>
+    <hyperlink ref="F17" r:id="rId11" xr:uid="{671646BC-4048-784B-A41A-EE3B6A5872DF}"/>
+    <hyperlink ref="H17" r:id="rId12" xr:uid="{520C3AB8-D98F-5A41-A791-18E65C05A26D}"/>
+    <hyperlink ref="I17" r:id="rId13" xr:uid="{AC194642-8CCA-D045-8B43-2E593C852C84}"/>
+    <hyperlink ref="K11" r:id="rId14" xr:uid="{7AD87150-852A-EC48-8A33-35899592670A}"/>
+    <hyperlink ref="I13" r:id="rId15" display="mailto:Jyin5@uoregon.edu" xr:uid="{BD89C2C8-01DA-0945-8C45-44FC2597E1A0}"/>
+    <hyperlink ref="I9" r:id="rId16" display="mailto:konao@uoregon.edu" xr:uid="{99A77FB4-F7EA-7A4E-A1D6-82B0846E355F}"/>
+    <hyperlink ref="K9" r:id="rId17" xr:uid="{72314501-811D-D043-997F-E392845F576D}"/>
+    <hyperlink ref="I3" r:id="rId18" xr:uid="{3B7DC98F-564E-8040-ABB3-24351F91CBD2}"/>
+    <hyperlink ref="G2" r:id="rId19" xr:uid="{944B277E-1502-DF4C-99EE-2856B2C13CD9}"/>
+    <hyperlink ref="I5" r:id="rId20" xr:uid="{645371C2-8065-1B4A-88CC-9620DE24CB5D}"/>
+    <hyperlink ref="K2" r:id="rId21" xr:uid="{9F15A558-4292-AB4D-AC30-3729FB430809}"/>
+    <hyperlink ref="I4" r:id="rId22" xr:uid="{A6D19378-1F6F-E544-8715-6F1C916ECD89}"/>
+    <hyperlink ref="I6" r:id="rId23" xr:uid="{1A222B28-25D7-3944-98F3-69D5F472A667}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3201,62 +3671,62 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" t="s">
         <v>116</v>
       </c>
-      <c r="B2" t="s">
-        <v>117</v>
-      </c>
       <c r="C2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -3277,7 +3747,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
@@ -3286,24 +3756,24 @@
         <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -3314,13 +3784,13 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -3328,16 +3798,16 @@
     </row>
     <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -3345,16 +3815,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E5">
         <v>2</v>
@@ -3362,16 +3832,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E6">
         <v>2</v>
@@ -3379,16 +3849,16 @@
     </row>
     <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -3396,16 +3866,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -3413,16 +3883,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -3433,13 +3903,13 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
+        <v>334</v>
+      </c>
+      <c r="C10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>335</v>
-      </c>
-      <c r="C10" t="s">
-        <v>122</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>